<commit_message>
Add direct text input/output support
</commit_message>
<xml_diff>
--- a/hasil_pengujian.xlsx
+++ b/hasil_pengujian.xlsx
@@ -977,10 +977,10 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>0.172486</v>
+        <v>0.184625</v>
       </c>
       <c r="E2" t="n">
-        <v>0.129467</v>
+        <v>0.188347</v>
       </c>
     </row>
     <row r="3">
@@ -998,10 +998,10 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>0.121733</v>
+        <v>0.183088</v>
       </c>
       <c r="E3" t="n">
-        <v>0.107086</v>
+        <v>0.166875</v>
       </c>
     </row>
     <row r="4">
@@ -1019,10 +1019,10 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>0.121792</v>
+        <v>0.171087</v>
       </c>
       <c r="E4" t="n">
-        <v>0.11272</v>
+        <v>0.385625</v>
       </c>
     </row>
     <row r="5">
@@ -1040,10 +1040,10 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>0.138144</v>
+        <v>0.221602</v>
       </c>
       <c r="E5" t="n">
-        <v>0.107984</v>
+        <v>0.188279</v>
       </c>
     </row>
     <row r="6">
@@ -1061,10 +1061,10 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>0.1189</v>
+        <v>0.22128</v>
       </c>
       <c r="E6" t="n">
-        <v>0.10801</v>
+        <v>0.223389</v>
       </c>
     </row>
     <row r="7">
@@ -1082,10 +1082,10 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>0.12992</v>
+        <v>0.258461</v>
       </c>
       <c r="E7" t="n">
-        <v>0.147196</v>
+        <v>0.202206</v>
       </c>
     </row>
   </sheetData>
@@ -1111,52 +1111,52 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>50.22935779816514</v>
+        <v>48.05045871559633</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>52.1788990825688</v>
+        <v>49.31192660550459</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>46.6743119266055</v>
+        <v>50.11467889908256</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>52.86697247706422</v>
+        <v>51.72018348623853</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>52.06422018348624</v>
+        <v>46.90366972477064</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>51.14678899082568</v>
+        <v>53.21100917431193</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>48.96788990825688</v>
+        <v>52.63761467889908</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>47.8211009174312</v>
+        <v>49.88532110091743</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>46.78899082568807</v>
+        <v>50.22935779816514</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>51.14678899082568</v>
+        <v>47.59174311926606</v>
       </c>
     </row>
   </sheetData>
@@ -1190,7 +1190,7 @@
         <v>4.04718240301417</v>
       </c>
       <c r="B2" t="n">
-        <v>7.925716133651568</v>
+        <v>7.908492245372438</v>
       </c>
     </row>
   </sheetData>

</xml_diff>